<commit_message>
cap nhat cac tinh nang de nghi bao hiem, kiem dinh taximet va the chap
</commit_message>
<xml_diff>
--- a/public/de_nghi_cap_bao_hiem_template.xlsx
+++ b/public/de_nghi_cap_bao_hiem_template.xlsx
@@ -4,28 +4,58 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Danh sách xe" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Bao_cao" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>TÊN CÔNG TY BẢO HIỂM:</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>DANH SÁCH XE HẾT HẠN BẢO HIỂM</t>
   </si>
   <si>
     <t>STT</t>
   </si>
   <si>
-    <t>Biển số xe</t>
-  </si>
-  <si>
-    <t>Ngày hết hạn cũ</t>
-  </si>
-  <si>
-    <t>Ghi chú</t>
+    <t>BIỂN SỐ</t>
+  </si>
+  <si>
+    <t>MÃ ĐÀM</t>
+  </si>
+  <si>
+    <t>LOẠI BẢO HIỂM</t>
+  </si>
+  <si>
+    <t>THỜI HẠN</t>
+  </si>
+  <si>
+    <t>SỐ ĐĂNG KÝ</t>
+  </si>
+  <si>
+    <t>SỐ KHUNG</t>
+  </si>
+  <si>
+    <t>SỐ MÁY</t>
+  </si>
+  <si>
+    <t>NHÃN HIỆU</t>
+  </si>
+  <si>
+    <t>NĂM SX</t>
+  </si>
+  <si>
+    <t>SỐ CHỖ</t>
+  </si>
+  <si>
+    <t>NƯỚC SX</t>
+  </si>
+  <si>
+    <t>NGÀY ĐĂNG KÝ XE LẦN ĐẦU</t>
+  </si>
+  <si>
+    <t>TÊN ĐĂNG KÝ XE</t>
   </si>
 </sst>
 </file>
@@ -47,20 +77,26 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -85,16 +121,16 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,24 +471,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="1" max="1" width="7.66" customWidth="1"/>
+    <col min="2" max="2" width="13.22" customWidth="1"/>
+    <col min="3" max="3" width="10.11" customWidth="1"/>
+    <col min="4" max="4" width="18.11" customWidth="1"/>
+    <col min="5" max="5" width="15.11" customWidth="1"/>
+    <col min="6" max="6" width="16.33" customWidth="1"/>
+    <col min="7" max="7" width="23.89" customWidth="1"/>
+    <col min="8" max="8" width="20.78" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="11.33" customWidth="1"/>
+    <col min="11" max="11" width="10.11" customWidth="1"/>
+    <col min="12" max="12" width="13.89" customWidth="1"/>
+    <col min="13" max="13" width="20.78" customWidth="1"/>
+    <col min="14" max="14" width="37.66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="25.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
     </row>
-    <row r="2" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" ht="22.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -465,18 +524,58 @@
       <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="4"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>